<commit_message>
Finalized first ad-hoc update
</commit_message>
<xml_diff>
--- a/auxiliary_data/Data_source_information.xlsx
+++ b/auxiliary_data/Data_source_information.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20411"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20416"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\meurerst\git\Anon-Lit-Review\eval_rev1\auxiliary_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\meurerst\git\anonymization-review\auxiliary_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A5C7AFA-EDED-4CDB-AF6B-74C8D9676E5B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3CB82D0-E31C-44E2-A755-34BB656953D1}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6756" yWindow="3096" windowWidth="23832" windowHeight="15552" xr2:uid="{5C5B0C05-51CD-4CF5-9CFB-2EAE4098E52C}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="26">
   <si>
     <t>Optum</t>
   </si>
@@ -54,9 +54,6 @@
     <t>NPS MedicineWise</t>
   </si>
   <si>
-    <t>Western Australian Data Linkage System</t>
-  </si>
-  <si>
     <t>TriNetX</t>
   </si>
   <si>
@@ -78,9 +75,6 @@
     <t>NPS</t>
   </si>
   <si>
-    <t>WADLS</t>
-  </si>
-  <si>
     <t>United States</t>
   </si>
   <si>
@@ -100,6 +94,15 @@
   </si>
   <si>
     <t>Origin (Data source)</t>
+  </si>
+  <si>
+    <t>InGef</t>
+  </si>
+  <si>
+    <t>Germany</t>
+  </si>
+  <si>
+    <t>IQVIA</t>
   </si>
 </sst>
 </file>
@@ -451,21 +454,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7335D3F3-4041-4819-94DB-544467FAE796}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
+    <col min="3" max="3" width="29.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" t="s">
         <v>22</v>
-      </c>
-      <c r="B1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C1" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
@@ -476,7 +480,7 @@
         <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
@@ -484,10 +488,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.3">
@@ -495,10 +499,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
@@ -506,10 +510,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
@@ -517,10 +521,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
@@ -528,10 +532,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C7" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
@@ -539,10 +543,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.3">
@@ -553,7 +557,7 @@
         <v>7</v>
       </c>
       <c r="C9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.3">
@@ -561,32 +565,43 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="B11" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="C11" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C12" t="s">
-        <v>18</v>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>